<commit_message>
Tweak to the pda description
</commit_message>
<xml_diff>
--- a/translate.xlsx
+++ b/translate.xlsx
@@ -1176,7 +1176,7 @@
     <t>EncyDesc_DrillTool</t>
   </si>
   <si>
-    <t>The Drill Tool is an industrial instrument capable of extracting mineral formations that are otherwise impenetrable by standard survival equipment.
+    <t>The drill tool is an industrial instrument capable of extracting mineral formations that are otherwise impenetrable by standard survival equipment.
 It allows for high-yield resource harvesting without the deployment of a Prawn Suit.
 - Reinforced industrial diamond coating enables fracturing the molecular bonds of large mineral veins
 - Rear-facing micro-thrusters prevent the operator from being propelled backward by the drill's resistance
@@ -1184,7 +1184,7 @@
 "By bypassing the need for heavy vehicular deployment, you have saved Alterra 4.2 credits in fuel cell depreciation. You're welcome."</t>
   </si>
   <si>
-    <t>Die Boorgereedskap is 'n industriële instrument wat in staat is om mineraalformasies te onttrek wat andersins ondeurdringbaar is deur standaard oorlewingstoerusting.
+    <t>Die boorgereedskap is 'n industriële instrument wat in staat is om mineraalformasies te onttrek wat andersins ondeurdringbaar is deur standaard oorlewingstoerusting.
 Dit maak voorsiening vir hoë-opbrengs hulpbron-oes sonder die ontplooiing van 'n Garnalepak.
 - Versterkte industriële diamantlaag maak dit moontlik om die molekulêre bindings van groot mineraalare te breek.
 - Agtertoe gerigte mikro-stuwers verhoed dat die operateur deur die boor se weerstand agtertoe gedryf word.
@@ -1203,52 +1203,52 @@
     <t>L'eina de perforació és un instrument industrial capaç d'extreure formacions minerals que d'altra banda serien impenetrables per a equips de supervivència estàndard.
 Permet la recobriment de recursos d'alt rendiment sense el desplegament d'un vestit de gamba.
 - El recobriment de diamant industrial reforçat permet fracturar els enllaços moleculars de grans venes minerals.
-- Els micropropulsors orientats cap enrere eviten que l'operador sigui impulsat cap enrere per la resistència del trepant.
-- El motor de parell variable ajusta les RPM en funció de la densitat del material per evitar que la broca s'enganxi i el rebot que pugui provocar una fractura del canell.
+- Els micropropulsors orientats cap enrere eviten que l'operador sigui impulsat cap enrere per la resistència de la perforadora.
+- El motor de parell variable ajusta les RPM en funció de la densitat del material per evitar que la broca s'enganxi i el rebot que es produeixi per fracturar el canell.
 "En evitar la necessitat de desplegament de vehicles pesats, heu estalviat a Alterra 4,2 crèdits en la depreciació de les piles de combustible. De res."</t>
   </si>
   <si>
-    <t>钻探工具是一种工业级仪器，能够开采标准生存装备无法穿透的矿层。
-它无需部署虾式机甲即可高效采集资源。
+    <t>这款钻机是一种工业级工具，能够开采标准生存装备无法穿透的矿层。
+它无需部署虾式机甲即可实现高产资源采集。
 - 强化型工业金刚石涂层能够破坏大型矿脉的分子键
-- 后置微型推进器可防止操作员因钻头阻力而被向后推
+- 后置微型推进器可防止操作员因钻机阻力而被向后推
 - 可变扭矩电机可根据材料密度调节转速，防止钻头卡死和手腕反冲
 “由于无需部署重型载具，您节省了 Alterra 4.2 点燃料电池折旧费用。不用谢。”</t>
   </si>
   <si>
-    <t>鑽探工具是一種工業級儀器，能夠開採標準生存裝備無法穿透的礦層。
-它無需部署蝦式機甲即可高效採集資源。
+    <t>這款鑽孔機是一種工業級工具，能夠開採標準生存裝備無法穿透的礦層。
+它無需部署蝦式機甲即可實現高產量資源採集。
 - 強化型工業用鑽石塗層能夠破壞大型礦脈的分子鍵
-- 後置微型推進器可防止操作員因鑽頭阻力而被向後推
+- 後置微型推進器可防止操作員因鑽機阻力而被向後推
 - 可變扭矩馬達可根據材料密度調節轉速，防止鑽頭卡死和手腕反轉
 “由於無需部署重型載具，您節省了 Alterra 4.2 點燃料電池折舊費用。不用謝。”</t>
   </si>
   <si>
     <t>Alat za bušenje je industrijski instrument sposoban za vađenje mineralnih formacija koje su inače neprobojne standardnom opremom za preživljavanje.
-Omogućuje visokoprinosno iskorištavanje resursa bez upotrebe Odijela za kozice.
+Omogućuje visokoprinosno iskorištavanje resursa bez upotrebe odijela za kozice.
 - Ojačani industrijski dijamantni premaz omogućuje razbijanje molekularnih veza velikih mineralnih žila
 - Mikro-potisnici okrenuti prema natrag sprječavaju da se operater pomiče unatrag otporom bušilice
 - Motor s promjenjivim momentom prilagođava broj okretaja na temelju gustoće materijala kako bi se spriječilo blokiranje svrdla i povratni udarac od loma ručnog zgloba
 "Zaobilaženjem potrebe za korištenjem teških vozila, uštedjeli ste Alterra 4,2 kredita u amortizaciji gorivnih ćelija. Nema na čemu."</t>
   </si>
   <si>
-    <t>Vrták je průmyslový nástroj schopný těžit minerální formace, které jsou jinak pro standardní vybavení pro přežití neproniknutelné.
-Umožňuje těžbu zdrojů s vysokým výtěžkem bez použití krevetového obleku.
+    <t>Vrtací nástroj je průmyslový nástroj schopný těžit minerální formace, které jsou jinak pro standardní vybavení pro přežití neproniknutelné.
+Umožňuje těžbu zdrojů s vysokým výtěžkem bez použití obleku Prawn Suit.
 - Zesílený průmyslový diamantový povlak umožňuje rozrušit molekulární vazby velkých minerálních žil.
 - Mikromotory směřující dozadu zabraňují tomu, aby byl obsluha hnána dozadu odporem vrtáku.
 - Motor s proměnným točivým momentem upravuje otáčky na základě hustoty materiálu, aby se zabránilo zaseknutí vrtáku a zpětnému rázu způsobenému zlomeninou zápěstí.
 „Tím, že jste se vyhnuli nutnosti nasazení těžkých vozidel, jste ušetřili 4,2 kreditu Alterra na odpisech palivových článků. Není zač.“</t>
   </si>
   <si>
-    <t>Drill Tool er et industrielt instrument, der er i stand til at udvinde mineralformationer, der ellers er uigennemtrængelige for standard overlevelsesudstyr.
+    <t>Boreværktøjet er et industrielt instrument, der er i stand til at udvinde mineralformationer, der ellers er uigennemtrængelige for standard overlevelsesudstyr.
 Det muliggør høst af ressourcer med højt udbytte uden brug af en rejedragt.
 - Forstærket industriel diamantbelægning muliggør brud på de molekylære bindinger i store mineralårer.
 - Bagudvendte mikro-thrustere forhindrer, at operatøren drives bagud af borets modstand.
-- Motor med variabelt moment justerer omdrejningstallet baseret på materialedensitet for at forhindre fastklemning af boret og tilbageslag fra håndledsbrud.
+- Motor med variabelt moment justerer omdrejningstallet baseret på materialedensitet for at forhindre borehovedbinding og tilbageslag fra håndledsbrud.
 "Ved at omgå behovet for tunge køretøjer har du sparet Alterra 4,2 point i afskrivning af brændstofceller. Velbekomme."</t>
   </si>
   <si>
-    <t>De boormachine is een industrieel instrument dat in staat is om minerale formaties te winnen die anders ondoordringbaar zijn voor standaard overlevingsuitrusting.
+    <t>De boor is een industrieel instrument dat in staat is om minerale formaties te winnen die anders ondoordringbaar zijn voor standaard overlevingsuitrusting.
 Het maakt een hoge opbrengst aan grondstoffenwinning mogelijk zonder de inzet van een Prawn Suit.
 - Versterkte industriële diamantcoating maakt het mogelijk om de moleculaire bindingen van grote minerale aderen te verbreken.
 - Naar achteren gerichte micro-stuwraketten voorkomen dat de operator door de weerstand van de boor naar achteren wordt geduwd.
@@ -1256,7 +1256,7 @@
 "Door de noodzaak van zwaar transport te omzeilen, heeft u Alterra 4,2 credits bespaard op de afschrijving van brandstofcellen. Graag gedaan."</t>
   </si>
   <si>
-    <t>Puurtööriist on tööstuslik instrument, mis on võimeline kaevandama mineraalkihte, mis muidu oleksid tavalise ellujäämisvarustusega läbimatud.
+    <t>See puurmasin on tööstuslik instrument, mis on võimeline kaevandama mineraalkihte, mis muidu oleksid tavalise ellujäämisvarustusega läbimatud.
 See võimaldab suure saagikusega ressursse koguda ilma krevetiülikonnata.
 - Tugevdatud tööstuslik teemantkate võimaldab purustada suurte mineraalisoonte molekulaarsidemeid.
 - Tahapoole suunatud mikromootorid takistavad operaatori tagasilööki puuri takistuse tõttu.
@@ -1264,19 +1264,19 @@
 "Raskete sõidukite kasutamise vajaduse vältimisega olete säästnud Alterrale 4,2 krediiti kütuseelementide amortisatsiooni pealt. Pole tänu väärt."</t>
   </si>
   <si>
-    <t>Porakone on teollisuuslaite, jolla voidaan louhia mineraalimuodostelmia, jotka muuten olisivat läpäisemättömiä tavallisilla selviytymisvarusteilla.
+    <t>Poraustyökalu on teollisuuslaite, jolla voidaan louhia mineraalimuodostelmia, jotka muuten olisivat läpäisemättömiä tavallisilla selviytymisvarusteilla.
 Se mahdollistaa suuren saannon luonnonvarojen keräämisen ilman katkarapuvun käyttöä.
 - Vahvistettu teollinen timanttipinnoite mahdollistaa suurten mineraalijuonien molekyylisidosten murtamisen.
-- Taaksepäin suunnatut mikropropulsiot estävät käyttäjää lennähtämästä taaksepäin poran vastuksen vaikutuksesta.
+- Taaksepäin suunnatut mikrotyöntövoimalaitteet estävät käyttäjää lennähtämästä taaksepäin poran vastuksen vaikutuksesta.
 - Muuttuvan vääntömomentin moottori säätää kierroslukua materiaalin tiheyden perusteella estääkseen terän juuttumisen ja ranteen murtuman aiheuttaman takapotkun.
 "Ohittamalla raskaiden ajoneuvojen käytön tarpeen olet säästänyt Alterralta 4,2 krediittiä polttokennojen poistoissa. Ole hyvä."</t>
   </si>
   <si>
     <t>L'outil de forage est un instrument industriel capable d'extraire des formations minérales inaccessibles aux équipements de survie classiques.
-Il permet une exploitation optimale des ressources sans nécessiter de combinaison spéciale.
+Il permet une exploitation à haut rendement des ressources sans nécessiter de combinaison spéciale.
 - Son revêtement diamant industriel renforcé permet de fracturer les liaisons moléculaires des grands filons minéraux.
 - Des micro-propulseurs arrière empêchent l'opérateur d'être repoussé par la résistance de la foreuse.
-- Son moteur à couple variable ajuste la vitesse de rotation en fonction de la densité du matériau afin d'éviter le blocage du foret et les risques de blessure au poignet.
+- Son moteur à couple variable ajuste la vitesse de rotation en fonction de la densité du matériau afin d'éviter le blocage du trépan et les risques de blessure au poignet.
 « En évitant le déploiement de véhicules lourds, vous avez permis à Alterra d'économiser 4,2 crédits en amortissement de la pile à combustible. De rien. »</t>
   </si>
   <si>
@@ -1288,8 +1288,8 @@
 „Durch den Verzicht auf schwere Fahrzeuge haben Sie Alterra 4.2 Credits für die Brennstoffzellenabschreibung eingespart. Gern geschehen.“</t>
   </si>
   <si>
-    <t>Το Εργαλείο Τρυπανιού είναι ένα βιομηχανικό όργανο ικανό να εξάγει ορυκτούς σχηματισμούς που διαφορετικά θα ήταν αδιαπέραστοι από τον τυπικό εξοπλισμό επιβίωσης.
-Επιτρέπει τη συγκομιδή πόρων υψηλής απόδοσης χωρίς την ανάπτυξη μιας Στολής Γαρίδας.
+    <t>Το εργαλείο τρυπανιού είναι ένα βιομηχανικό όργανο ικανό να εξάγει ορυκτούς σχηματισμούς που διαφορετικά θα ήταν αδιαπέραστοι από τον τυπικό εξοπλισμό επιβίωσης.
+Επιτρέπει τη συγκομιδή πόρων υψηλής απόδοσης χωρίς την ανάπτυξη μιας στολής γαρίδας.
 - Η ενισχυμένη βιομηχανική επίστρωση διαμαντιού επιτρέπει τη θραύση των μοριακών δεσμών μεγάλων ορυκτών φλεβών
 - Οι μικρο-προωθητήρες που είναι στραμμένοι προς τα πίσω εμποδίζουν τον χειριστή να ωθηθεί προς τα πίσω από την αντίσταση του τρυπανιού
 - Ο κινητήρας μεταβλητής ροπής ρυθμίζει τις στροφές ανά λεπτό με βάση την πυκνότητα του υλικού για να αποτρέψει το μπλοκάρισμα του τρυπανιού και το κλώτσημα από το κάταγμα του καρπού
@@ -1304,23 +1304,23 @@
 "A nehéz járművek használatának megkerülésével 4,2 kreditet takarított meg az Alterra üzemanyagcella-értékcsökkenésén. Szívesen."</t>
   </si>
   <si>
-    <t>Is uirlis thionsclaíoch í an Uirlis Druileála atá in ann foirmíochtaí mianraí a bhaint amach nach mbeadh trealaimh mharthanais chaighdeánacha in ann dul tríd murach sin.
-Ceadaíonn sé fómhar acmhainní ard-toraidh gan Culaith Cloicheán a imscaradh.
+    <t>Is uirlis thionsclaíoch í an uirlis druileála atá in ann foirmíochtaí mianraí a bhaint amach nach mbeadh trealaimh mharthanais chaighdeánacha in ann dul tríd murach sin.
+Ceadaíonn sé fómhar acmhainní ard-toraidh gan úsáid a bhaint as Culaith Cloicheán.
 - Cumasaíonn sciath diamant tionsclaíoch athneartaithe naisc mhóilíneacha féitheacha móra mianraí a bhriseadh
 - Coscann micrea-bhrúiteoirí atá os comhair an chúl an t-oibreoir ó bheith á thiomáint siar ag friotaíocht an druileála
 - Coigeartaíonn mótar chasmhóiminte athraitheach RPM bunaithe ar dhlús ábhair chun ceangal giotán agus cic siar briste caol na láimhe a chosc
-"Tríd an ngá atá le himscaradh feithiclí troma a sheachaint, tá 4.2 creidiúint Alterra sábháilte agat i ndíluacháil cealla breosla. Tá fáilte romhat."</t>
+"Tríd an ngá atá le húsáid feithiclí troma a sheachaint, tá 4.2 creidiúint Alterra sábháilte agat i ndíluacháil cealla breosla. Tá fáilte romhat."</t>
   </si>
   <si>
     <t>La trivella è uno strumento industriale in grado di estrarre formazioni minerarie altrimenti impenetrabili con le normali attrezzature di sopravvivenza.
-Consente l'estrazione di risorse ad alto rendimento senza la necessità di indossare una tuta Prawn.
+Consente un'estrazione di risorse ad alto rendimento senza la necessità di indossare una tuta Prawn.
 - Il rivestimento diamantato industriale rinforzato permette di fratturare i legami molecolari di grandi vene minerarie.
 - I micro-propulsori posteriori impediscono all'operatore di essere spinto all'indietro dalla resistenza della trivella.
 - Il motore a coppia variabile regola i giri al minuto in base alla densità del materiale per evitare l'inceppamento della punta e il contraccolpo che potrebbe causare fratture al polso.
 "Evitando l'impiego di veicoli pesanti, hai risparmiato 4,2 crediti Alterra in ammortamento delle celle a combustibile. Prego."</t>
   </si>
   <si>
-    <t>ドリルツールは、通常のサバイバル装備では掘削不可能な鉱物層を採掘できる産業用機器です。
+    <t>このドリルツールは、通常のサバイバル装備では掘削不可能な鉱物層を採掘できる産業用機器です。
 これにより、プラウンスーツを装備することなく、高収量の資源採掘が可能になります。
 - 強化された工業用ダイヤモンドコーティングにより、大型鉱脈の分子結合を破壊します。
 - 後方に取り付けられたマイクロスラスタにより、ドリルの抵抗によってオペレーターが後方に押し戻されるのを防ぎます。
@@ -1328,8 +1328,8 @@
 「大型車両の展開が不要になったことで、燃料電池の減価償却費をアルテラ4.2クレジット節約できました。どういたしまして。」</t>
   </si>
   <si>
-    <t>드릴 툴은 일반적인 생존 장비로는 접근할 수 없는 광물층을 채굴할 수 있는 산업용 장비입니다.
-프론 슈트를 착용하지 않고도 높은 수확량의 자원을 채취할 수 있습니다.
+    <t>드릴 도구는 일반적인 생존 장비로는 접근할 수 없는 광물층을 채굴할 수 있는 산업용 장비입니다.
+프론 슈트(Prawn Suit)를 착용하지 않고도 높은 수확량의 자원을 채취할 수 있습니다.
 - 강화된 산업용 다이아몬드 코팅으로 대형 광맥의 분자 결합을 파괴할 수 있습니다.
 - 후방 마이크로 추진기는 드릴의 저항으로 인해 작업자가 뒤로 밀리지 않도록 방지합니다.
 - 가변 토크 모터는 재료 밀도에 따라 회전수를 조절하여 드릴 비트 걸림과 손목 골절을 방지합니다.
@@ -1341,7 +1341,7 @@
 - Pastiprināts rūpnieciskais dimanta pārklājums ļauj pārraut lielu minerālu vēnu molekulārās saites.
 - Aizmugurē vērsti mikrodzinēji neļauj operatoram tikt atgrūstam atpakaļ urbja pretestības dēļ.
 - Mainīga griezes momenta motors pielāgo apgriezienus minūtē, pamatojoties uz materiāla blīvumu, lai novērstu urbja iesprūšanu un plaukstas locītavas lūzuma atsitienu.
-"Apejot nepieciešamību izmantot smagus transportlīdzekļus, jūs esat ietaupījis Alterra 4,2 kredītpunktus degvielas elementu nolietojumā. Nav par ko."</t>
+"Apejot nepieciešamību izmantot smagos transportlīdzekļus, jūs esat ietaupījis Alterra 4,2 kredītpunktus degvielas elementu nolietojumā. Nav par ko."</t>
   </si>
   <si>
     <t>Gręžimo įrankis yra pramoninis instrumentas, galintis išgauti mineralinius darinius, į kuriuos kitaip neįsibrautų standartinė išgyvenimo įranga.
@@ -1349,27 +1349,27 @@
 - Sustiprinta pramoninė deimantinė danga leidžia suardyti didelių mineralinių gyslų molekulinius ryšius.
 - Galiniai mikrovarikliai neleidžia operatoriui būti stumtam atgal dėl grąžto pasipriešinimo.
 - Kintamo sukimo momento variklis reguliuoja apsukas pagal medžiagos tankį, kad būtų išvengta grąžto strigimo ir riešo lūžio atatrankos.
-„Aplenkdami poreikį naudoti sunkias transporto priemones, sutaupėte 4,2 „Alterra“ kreditų už kuro elementų nusidėvėjimą. Prašom.“</t>
-  </si>
-  <si>
-    <t>Drill Tool er et industrielt instrument som er i stand til å utvinne mineralformasjoner som ellers er ugjennomtrengelige med standard overlevelsesutstyr.
+„Aplenkdami poreikį naudoti sunkiasvores transporto priemones, sutaupėte 4,2 „Alterra“ kreditų už kuro elementų nusidėvėjimą. Prašom.“</t>
+  </si>
+  <si>
+    <t>Boreverktøyet er et industrielt instrument som er i stand til å utvinne mineralformasjoner som ellers er ugjennomtrengelige med standard overlevelsesutstyr.
 Det muliggjør høyavkastende ressurshøsting uten bruk av rekedrakt.
 - Forsterket industrielt diamantbelegg muliggjør brudd i de molekylære bindingene i store mineralårer.
 - Bakovervendte mikro-thrustere forhindrer at operatøren drives bakover av borets motstand.
-- Variabelt dreiemomentmotor justerer turtallet basert på materialtetthet for å forhindre at boret setter seg fast og tilbakeslag som kan forårsake håndleddsbrudd.
-"Ved å omgå behovet for tunge kjøretøy, har du spart Alterra 4,2 studiepoeng i avskrivning av brenselceller. Bare hyggelig."</t>
-  </si>
-  <si>
-    <t>Drill Tool to narzędzie przemysłowe, które umożliwia wydobywanie z formacji mineralnych, które są w innym przypadku niedostępne dla standardowego sprzętu survivalowego.
+- Motor med variabelt dreiemoment justerer turtallet basert på materialtetthet for å forhindre at boret setter seg fast og tilbakeslag som kan forårsake håndleddsbrudd.
+"Ved å omgå behovet for bruk av tunge kjøretøy har du spart Alterra 4,2 studiepoeng i avskrivning av brenselceller. Bare hyggelig."</t>
+  </si>
+  <si>
+    <t>Wiertnica to urządzenie przemysłowe, które umożliwia wydobywanie z formacji mineralnych, które są w innym przypadku niedostępne dla standardowego sprzętu survivalowego.
 Umożliwia ono wysokowydajne pozyskiwanie surowców bez użycia kombinezonu Prawn.
 - Wzmocniona przemysłowa powłoka diamentowa umożliwia rozrywanie wiązań molekularnych w dużych żyłach mineralnych.
-- Mikrosilniki skierowane do tyłu zapobiegają odpychaniu operatora do tyłu przez opór wiertła.
+- Mikrosilniki skierowane do tyłu zapobiegają odpychaniu operatora do tyłu przez opór wiertarki.
 - Silnik o zmiennym momencie obrotowym dostosowuje obroty na podstawie gęstości materiału, aby zapobiec zakleszczaniu się wiertła i odrzutowi nadgarstka.
-„Dzięki wyeliminowaniu konieczności użycia ciężkich pojazdów zaoszczędziłeś firmie Alterra 4,2 punktu na amortyzacji ogniw paliwowych. Zapraszamy”.</t>
-  </si>
-  <si>
-    <t>A Ferramenta de Perfuração é um instrumento industrial capaz de extrair formações minerais que seriam impenetráveis ​​para equipamentos de sobrevivência padrão.
-Ela permite a extração de recursos de alto rendimento sem a necessidade de usar um Traje PRAWN.
+„Dzięki wyeliminowaniu konieczności użycia ciężkich pojazdów zaoszczędziliście Państwo firmie Alterra 4,2 kredytu na amortyzacji ogniw paliwowych. Zapraszamy”.</t>
+  </si>
+  <si>
+    <t>A ferramenta de perfuração é um instrumento industrial capaz de extrair formações minerais que seriam impenetráveis ​​para equipamentos de sobrevivência padrão.
+Ela permite a extração de recursos de alto rendimento sem a necessidade de usar um traje PRAWN.
 - O revestimento reforçado de diamante industrial permite fraturar as ligações moleculares de grandes veios minerais.
 - Micropropulsores traseiros impedem que o operador seja impulsionado para trás pela resistência da perfuratriz.
 - O motor de torque variável ajusta a RPM com base na densidade do material para evitar o travamento da broca e o recuo que pode causar fraturas no pulso.
@@ -1379,7 +1379,7 @@
     <t>Instrumentul de foraj este un instrument industrial capabil să extragă formațiuni minerale care altfel ar fi impenetrabile de echipamentele standard de supraviețuire.
 Permite recoltarea resurselor cu randament ridicat fără a fi nevoie de utilizarea unui costum Prawn.
 - Stratul industrial ranforsat cu diamant permite fracturarea legăturilor moleculare ale venelor minerale mari
-- Micropropulsoarele orientate spre spate împiedică operatorul să fie propulsat înapoi de rezistența burghiului
+- Micropropulsoarele orientate spre spate împiedică operatorul să fie propulsat înapoi de rezistența forajului
 - Motorul cu cuplu variabil ajustează turația în funcție de densitatea materialului pentru a preveni blocarea burghiului și reculul cauzat de fracturarea încheieturii mâinii
 „Evitând necesitatea utilizării vehiculelor grele, ați economisit 4,2 credite la Alterra în deprecierea pilelor de combustibil. Cu plăcere.”</t>
   </si>
@@ -1397,10 +1397,10 @@
 - Ојачани индустријски дијамантски премаз омогућава разбијање молекуларних веза великих минералних вена.
 - Микро-потисници окренути уназад спречавају да оператер буде потиснут уназад отпором бушилице.
 - Мотор са променљивим обртним моментом подешава број обртаја на основу густине материјала како би се спречило заглављивање бургије и повратни ударац услед прелома зглоба.
-„Заобилажењем потребе за тешким возилима, уштедели сте Алтери 4,2 кредита у амортизацији горивних ћелија. Нема на чему.“</t>
-  </si>
-  <si>
-    <t>Vŕtačka je priemyselný nástroj schopný ťažiť minerálne formácie, ktoré sú inak nepreniknuteľné štandardným vybavením na prežitie.
+„Заобилажењем потребе за распоређивањем тешких возила, уштедели сте Алтери 4,2 кредита у амортизацији горивних ћелија. Нема на чему.“</t>
+  </si>
+  <si>
+    <t>Vŕtací nástroj je priemyselný nástroj schopný ťažiť minerálne formácie, ktoré sú inak nepreniknuteľné štandardným vybavením na prežitie.
 Umožňuje ťažbu zdrojov s vysokým výnosom bez použitia krevetového obleku.
 - Zosilnený priemyselný diamantový povlak umožňuje rozbíjanie molekulárnych väzieb veľkých minerálnych žíl
 - Mikromotory smerujúce dozadu zabraňujú tomu, aby bol operátor hnaný dozadu odporom vrtáka
@@ -1408,7 +1408,7 @@
 „Vďaka obídeniu potreby nasadenia ťažkých vozidiel ste ušetrili 4,2 kreditu Alterra na odpisoch palivových článkov. Nie je zač.“</t>
   </si>
   <si>
-    <t>Vrtalno orodje je industrijski instrument, ki lahko izkopava mineralne formacije, ki so sicer neprebojne za standardno opremo za preživetje.
+    <t>Vrtalno orodje je industrijski instrument, ki lahko izkopava mineralne formacije, ki so sicer neprebojne s standardno opremo za preživetje.
 Omogoča visoko donosno pridobivanje virov brez uporabe zaščitne obleke za kozice.
 - Ojačana industrijska diamantna prevleka omogoča lomljenje molekularnih vezi velikih mineralnih žil.
 - Mikropotisniki, obrnjeni nazaj, preprečujejo, da bi upor svedra potisnil upravljavca nazaj.
@@ -1416,20 +1416,20 @@
 "Z izogibanjem potrebi po uporabi težkih vozil ste prihranili 4,2 kreditne točke Alterra pri amortizaciji gorivnih celic. Ni za kaj."</t>
   </si>
   <si>
-    <t>La Perforadora es un instrumento industrial capaz de extraer formaciones minerales impenetrables para el equipo de supervivencia estándar.
+    <t>La herramienta de perforación es un instrumento industrial capaz de extraer formaciones minerales impenetrables para el equipo de supervivencia estándar.
 Permite la extracción de recursos de alto rendimiento sin necesidad de usar un traje Prawn.
-- El revestimiento reforzado de diamante industrial permite fracturar los enlaces moleculares de grandes vetas minerales.
-- Los micropropulsores traseros evitan que el operador retroceda debido a la resistencia de la perforadora.
+- El recubrimiento reforzado de diamante industrial permite fracturar los enlaces moleculares de grandes vetas minerales.
+- Los micropropulsores traseros evitan que el operador retroceda debido a la resistencia de la perforación.
 - El motor de par variable ajusta las RPM según la densidad del material para evitar que la broca se atasque y el retroceso por fractura de muñeca.
 "Al evitar la necesidad de desplegar vehículos pesados, le has ahorrado a Alterra 4.2 créditos en depreciación de celdas de combustible. De nada."</t>
   </si>
   <si>
     <t>Borrverktyget är ett industriellt instrument som kan utvinna mineralformationer som annars är ogenomträngliga med vanlig överlevnadsutrustning.
-Det möjliggör högavkastande resursutvinning utan att en räkdräkt behöver användas.
+Det möjliggör högavkastande resursutvinning utan användning av räkdräkt.
 - Förstärkt industriell diamantbeläggning möjliggör spräckning av de molekylära bindningarna i stora mineralådror.
 - Bakåtvända mikromotorer förhindrar att operatören drivs bakåt av borrens motstånd.
 - Motor med variabelt vridmoment justerar varvtalet baserat på materialdensitet för att förhindra att borren fastnar och kast som orsakar handledsfrakturer.
-"Genom att undvika behovet av tunga fordon har du sparat Alterra 4,2 poäng i bränslecellsavskrivning. Varsågod."</t>
+"Genom att kringgå behovet av tunga fordon har du sparat Alterra 4,2 poäng i bränslecellsavskrivning. Varsågod."</t>
   </si>
   <si>
     <t>เครื่องมือเจาะนี้เป็นเครื่องมืออุตสาหกรรมที่สามารถสกัดแร่ธาตุที่อุปกรณ์เอาชีวิตรอดมาตรฐานไม่สามารถเข้าถึงได้
@@ -1440,20 +1440,20 @@
 "ด้วยการหลีกเลี่ยงความจำเป็นในการใช้ยานพาหนะขนาดใหญ่ คุณได้ประหยัดค่าเสื่อมราคาของเซลล์เชื้อเพลิงให้กับ Alterra ไป 4.2 เครดิต ยินดีครับ"</t>
   </si>
   <si>
-    <t>Matkap Aleti, standart hayatta kalma ekipmanlarıyla geçilemeyen mineral oluşumlarını çıkarabilen endüstriyel bir alettir.
+    <t>Bu matkap, standart hayatta kalma ekipmanlarıyla geçilemeyen mineral oluşumlarını çıkarabilen endüstriyel bir alettir.
 Bir Prawn Suit'in kullanılmasına gerek kalmadan yüksek verimli kaynak hasadı sağlar.
 - Güçlendirilmiş endüstriyel elmas kaplama, büyük mineral damarlarının moleküler bağlarını kırmayı sağlar.
 - Arkaya bakan mikro iticiler, operatörün matkabın direncinden dolayı geriye doğru itilmesini önler.
-- Değişken torklu motor, uç sıkışmasını ve bilek kırılmasına neden olabilecek geri tepmeyi önlemek için devir sayısını malzeme yoğunluğuna göre ayarlar.
+- Değişken torklu motor, uç sıkışmasını ve bilek kırılmasına neden olabilecek geri tepmeyi önlemek için malzeme yoğunluğuna göre devir sayısını ayarlar.
 "Ağır araç kullanımına gerek kalmadan, Alterra'nın yakıt hücresi amortismanında 4,2 kredi tasarruf sağladınız. Rica ederim."</t>
   </si>
   <si>
-    <t>Буровий інструмент – це промисловий інструмент, здатний видобувати мінеральні утворення, які інакше непроникні для стандартного спорядження для виживання.
+    <t>Буровий інструмент — це промисловий інструмент, здатний видобувати мінеральні утворення, які інакше непроникні для стандартного спорядження для виживання.
 Він дозволяє видобувати високопродуктивні ресурси без використання костюма для креветок.
 - Посилене промислове алмазне покриття дозволяє руйнувати молекулярні зв'язки великих мінеральних жил.
 - Мікродвигуни, спрямовані назад, запобігають відкиданню оператора назад опором бура.
 - Двигун зі змінним крутним моментом регулює швидкість обертання залежно від щільності матеріалу, щоб запобігти заклинюванню долота та віддачі від перелому зап'ястя.
-"Уникаючи необхідності використання важкого транспортного засобу, ви заощадили 4,2 кредити Alterra на амортизації паливних елементів. Будь ласка."</t>
+«Уникаючи необхідності використання важкого транспортного засобу, ви заощадили 4,2 кредити Alterra на амортизації паливних елементів. Будь ласка».</t>
   </si>
   <si>
     <t>Máy khoan là một thiết bị công nghiệp có khả năng khai thác các mỏ khoáng sản mà các thiết bị sinh tồn tiêu chuẩn không thể tiếp cận được.

</xml_diff>

<commit_message>
fix issue for the translate key, also the pda and blueprint popups are working
</commit_message>
<xml_diff>
--- a/translate.xlsx
+++ b/translate.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="391">
   <si>
     <t>Keycode</t>
   </si>
@@ -574,6 +574,9 @@
     <t>Hitinterval</t>
   </si>
   <si>
+    <t>Interval raken</t>
+  </si>
+  <si>
     <t>Tabamuse intervall</t>
   </si>
   <si>
@@ -670,12 +673,12 @@
 Utilitzeu el valor per defecte per coincidir amb la velocitat de mineria d'un braç perforador amb vestit de gambes.</t>
   </si>
   <si>
-    <t>资源矿藏的采集间隔。
+    <t>资源矿脉的采集间隔。
 间隔越小，采集速度越快。
 使用默认值以匹配虾式机甲钻臂的采矿速度。</t>
   </si>
   <si>
-    <t>資源礦藏的採集間隔。
+    <t>資源礦脈的採集間隔。
 間隔越小，採集速度越快。
 使用預設值以匹配蝦式機甲鑽臂的採礦速度。</t>
   </si>
@@ -1161,16 +1164,31 @@
     <t>Ency_DrillTool</t>
   </si>
   <si>
+    <t>Drill Tool</t>
+  </si>
+  <si>
     <t>Инструмент за пробиване</t>
   </si>
   <si>
     <t>Bohrwerkzeug</t>
   </si>
   <si>
+    <t>Uirlis Druileála</t>
+  </si>
+  <si>
+    <t>Utensile da trapano</t>
+  </si>
+  <si>
+    <t>Urbšanas rīks</t>
+  </si>
+  <si>
     <t>Сверло</t>
   </si>
   <si>
-    <t>Matkap aleti</t>
+    <t>Orodje za vrtanje</t>
+  </si>
+  <si>
+    <t>Matkap Aleti</t>
   </si>
   <si>
     <t>EncyDesc_DrillTool</t>
@@ -1241,10 +1259,10 @@
   </si>
   <si>
     <t>Boreværktøjet er et industrielt instrument, der er i stand til at udvinde mineralformationer, der ellers er uigennemtrængelige for standard overlevelsesudstyr.
-Det muliggør høst af ressourcer med højt udbytte uden brug af en rejedragt.
+Det muliggør høst af ressourcer med højt udbytte uden brug af rejedragt.
 - Forstærket industriel diamantbelægning muliggør brud på de molekylære bindinger i store mineralårer.
 - Bagudvendte mikro-thrustere forhindrer, at operatøren drives bagud af borets modstand.
-- Motor med variabelt moment justerer omdrejningstallet baseret på materialedensitet for at forhindre borehovedbinding og tilbageslag fra håndledsbrud.
+- Motor med variabelt moment justerer omdrejningstallet baseret på materialedensitet for at forhindre fastklemning af boret og tilbageslag fra håndledsbrud.
 "Ved at omgå behovet for tunge køretøjer har du sparet Alterra 4,2 point i afskrivning af brændstofceller. Velbekomme."</t>
   </si>
   <si>
@@ -1322,7 +1340,7 @@
   <si>
     <t>このドリルツールは、通常のサバイバル装備では掘削不可能な鉱物層を採掘できる産業用機器です。
 これにより、プラウンスーツを装備することなく、高収量の資源採掘が可能になります。
-- 強化された工業用ダイヤモンドコーティングにより、大型鉱脈の分子結合を破壊します。
+- 強化された工業用ダイヤモンドコーティングにより、大きな鉱脈の分子結合を破壊します。
 - 後方に取り付けられたマイクロスラスタにより、ドリルの抵抗によってオペレーターが後方に押し戻されるのを防ぎます。
 - 可変トルクモーターは、材料の密度に応じて回転数を調整し、ビットの詰まりや手首の骨折につながるキックバックを防ぎます。
 「大型車両の展開が不要になったことで、燃料電池の減価償却費をアルテラ4.2クレジット節約できました。どういたしまして。」</t>
@@ -1348,8 +1366,8 @@
 Jis leidžia išgauti didelį išteklių derlių nenaudojant krevečių kostiumo.
 - Sustiprinta pramoninė deimantinė danga leidžia suardyti didelių mineralinių gyslų molekulinius ryšius.
 - Galiniai mikrovarikliai neleidžia operatoriui būti stumtam atgal dėl grąžto pasipriešinimo.
-- Kintamo sukimo momento variklis reguliuoja apsukas pagal medžiagos tankį, kad būtų išvengta grąžto strigimo ir riešo lūžio atatrankos.
-„Aplenkdami poreikį naudoti sunkiasvores transporto priemones, sutaupėte 4,2 „Alterra“ kreditų už kuro elementų nusidėvėjimą. Prašom.“</t>
+- Kintamo sukimo momento variklis reguliuoja apsukas pagal medžiagos tankį, kad būtų išvengta grąžto užstrigimo ir riešo lūžio atatrankos.
+„Aplenkdami poreikį naudoti sunkias transporto priemones, sutaupėte 4,2 „Alterra“ kreditų už kuro elementų nusidėvėjimą. Prašom.“</t>
   </si>
   <si>
     <t>Boreverktøyet er et industrielt instrument som er i stand til å utvinne mineralformasjoner som ellers er ugjennomtrengelige med standard overlevelsesutstyr.
@@ -2633,587 +2651,587 @@
         <v>164</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P5" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q5" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R5" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S5" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T5" s="14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="X5" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="Y5" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Z5" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AA5" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AB5" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AC5" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AD5" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AE5" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AF5" s="14" t="s">
         <v>163</v>
       </c>
       <c r="AG5" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AH5" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AI5" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AJ5" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AK5" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AL5" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AM5" s="14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AN5" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="T6" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="W6" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="X6" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z6" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AC6" s="15" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AD6" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AE6" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AF6" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AG6" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AH6" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AI6" s="15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AJ6" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AK6" s="8" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AL6" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AM6" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AN6" s="17" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K7" s="14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N7" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="R7" s="14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="S7" s="14" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="T7" s="14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U7" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="V7" s="14" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="W7" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="X7" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Y7" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="Z7" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AA7" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AB7" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AC7" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AD7" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AE7" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AF7" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG7" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AH7" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AI7" s="15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AJ7" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AK7" s="14" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AL7" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="AM7" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AN7" s="16" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="N8" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P8" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q8" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="R8" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="T8" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="U8" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="V8" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="W8" s="8" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="X8" s="8" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Y8" s="8" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="Z8" s="8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AA8" s="8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="AC8" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="AD8" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AE8" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AF8" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="AG8" s="8" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="AH8" s="8" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="AI8" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="AJ8" s="8" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AK8" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AL8" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AM8" s="8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="AN8" s="17" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="O9" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="P9" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="Q9" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="R9" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="S9" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="T9" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="U9" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="V9" s="14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="W9" s="14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="X9" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Y9" s="14" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="Z9" s="14" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AA9" s="14" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AB9" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AC9" s="14" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="AD9" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AE9" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AF9" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="AG9" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="AH9" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AI9" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AJ9" s="14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="AK9" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AL9" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AM9" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AN9" s="16" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>40</v>
@@ -3270,7 +3288,7 @@
         <v>40</v>
       </c>
       <c r="T10" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="U10" s="8" t="s">
         <v>40</v>
@@ -3335,246 +3353,246 @@
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>229</v>
+        <v>345</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N11" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O11" s="14" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="P11" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q11" s="14" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="R11" s="14" t="s">
-        <v>245</v>
+        <v>348</v>
       </c>
       <c r="S11" s="14" t="s">
-        <v>246</v>
+        <v>349</v>
       </c>
       <c r="T11" s="14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U11" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="V11" s="14" t="s">
-        <v>249</v>
+        <v>350</v>
       </c>
       <c r="W11" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="X11" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Y11" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="Z11" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AA11" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AB11" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AC11" s="14" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="AD11" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AE11" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AF11" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG11" s="14" t="s">
-        <v>258</v>
+        <v>352</v>
       </c>
       <c r="AH11" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AI11" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AJ11" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AK11" s="14" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AL11" s="14" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="AM11" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AN11" s="16" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="18" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="I12" s="21" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="J12" s="21" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="L12" s="21" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="M12" s="21" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="N12" s="21" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="O12" s="21" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="P12" s="21" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="Q12" s="21" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="R12" s="21" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="S12" s="21" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="T12" s="21" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="U12" s="21" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="V12" s="21" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="W12" s="21" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="X12" s="21" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="Y12" s="21" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="Z12" s="21" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="AA12" s="21" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="AB12" s="21" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="AC12" s="21" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="AD12" s="21" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="AE12" s="21" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="AF12" s="21" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="AG12" s="21" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="AH12" s="21" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="AI12" s="21" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="AJ12" s="21" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="AK12" s="21" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="AL12" s="21" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="AM12" s="21" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="AN12" s="22" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
added auto collect localization
</commit_message>
<xml_diff>
--- a/translate.xlsx
+++ b/translate.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="462">
   <si>
     <t>Keycode</t>
   </si>
@@ -460,8 +460,8 @@
 エネルギーは、大規模な資源鉱床を採掘する場合にのみ消費されます。</t>
   </si>
   <si>
-    <t>자원 매장지 채굴 시 배터리 소모량이 발생합니다.
-매장지를 완전히 파괴하려면 최대 320번의 채굴이 필요합니다.
+    <t>자원 매장지 채굴 시마다 배터리가 소모됩니다.
+매장지를 완전히 파괴하려면 최대 320번 채굴해야 합니다.
 에너지는 대형 자원 매장지를 채굴할 때만 소모됩니다.</t>
   </si>
   <si>
@@ -574,6 +574,9 @@
     <t>Hitinterval</t>
   </si>
   <si>
+    <t>Interval raken</t>
+  </si>
+  <si>
     <t>Tabamuse intervall</t>
   </si>
   <si>
@@ -670,12 +673,12 @@
 Utilitzeu el valor per defecte per coincidir amb la velocitat de mineria d'un braç perforador amb vestit de gambes.</t>
   </si>
   <si>
-    <t>资源矿藏的采集间隔。
+    <t>资源矿脉的采集间隔。
 间隔越小，采集速度越快。
 使用默认值以匹配虾式机甲钻臂的采矿速度。</t>
   </si>
   <si>
-    <t>資源礦藏的採集間隔。
+    <t>資源礦脈的採集間隔。
 間隔越小，採集速度越快。
 使用預設值以匹配蝦式機甲鑽臂的採礦速度。</t>
   </si>
@@ -906,7 +909,7 @@
     <t>Vrtalno orodje</t>
   </si>
   <si>
-    <t>Herramienta de perforación</t>
+    <t>Taladro</t>
   </si>
   <si>
     <t>Taladro de mano</t>
@@ -1180,9 +1183,6 @@
   </si>
   <si>
     <t>Сверло</t>
-  </si>
-  <si>
-    <t>Taladro</t>
   </si>
   <si>
     <t>Matkap Aleti</t>
@@ -1219,14 +1219,14 @@
 "En evitar la necessitat de desplegament de vehicles pesats, heu estalviat a Alterra 4,2 crèdits en la depreciació de les piles de combustible. De res."</t>
   </si>
   <si>
-    <t>这款钻探工具是一种工业级仪器，无需使用虾式机甲，即可开采标准生存装备无法穿透的矿层。
+    <t>这台钻机是一种工业级仪器，无需使用虾式机甲，即可开采标准生存装备无法穿透的矿层。
 - 强化型工业金刚石涂层能够破坏大型矿脉的分子键
 - 后置微型推进器可防止操作员因钻头阻力而被向后推
 - 可变扭矩电机可根据材料密度调节转速，防止钻头卡死和手腕反冲
 “由于无需部署重型载具，您节省了 Alterra 4.2 点燃料电池折旧费用。不用谢。”</t>
   </si>
   <si>
-    <t>這款鑽探工具是一種工業級儀器，無需使用蝦式機甲，即可開採標準生存裝備無法穿透的礦層。
+    <t>這台鑽孔機是一種工業級儀器，無需使用蝦式機甲，即可開採標準生存裝備無法穿透的礦層。
 - 強化型工業用鑽石塗層能夠破壞大型礦脈的分子鍵
 - 後置微型推進器可防止操作員因鑽頭阻力而被向後推
 - 可變扭矩馬達可根據材料密度調節轉速，防止鑽頭卡死和手腕反轉
@@ -1240,10 +1240,10 @@
 "Zaobilaženjem potrebe za korištenjem teških vozila, uštedjeli ste Alterra 4,2 kredita u amortizaciji gorivnih ćelija. Nema na čemu."</t>
   </si>
   <si>
-    <t>Vrtací nástroj je průmyslový nástroj schopný těžit minerální formace, které jsou jinak pro standardní vybavení pro přežití neproniknutelné, a to bez použití obleku Prawn Suit.
+    <t>Vrtací nástroj je průmyslový nástroj schopný těžit minerální formace, které jsou jinak neproniknutelné standardním vybavením pro přežití, a to bez použití obleku Prawn Suit.
 - Zesílený průmyslový diamantový povlak umožňuje rozrušit molekulární vazby velkých minerálních žil.
 - Mikromotory směřující dozadu zabraňují tomu, aby byl obsluha hnána dozadu odporem vrtáku.
-- Motor s proměnným točivým momentem upravuje otáčky na základě hustoty materiálu, aby se zabránilo zaseknutí vrtáku a zpětnému rázu způsobujícímu zlomeninu zápěstí.
+- Motor s proměnným točivým momentem upravuje otáčky na základě hustoty materiálu, aby se zabránilo zaseknutí vrtáku a zpětnému rázu způsobenému zlomeninou zápěstí.
 „Tím, že jste se vyhnuli nutnosti nasazení těžkých vozidel, jste ušetřili 4,2 kreditu Alterra na odpisech palivových článků. Není zač.“</t>
   </si>
   <si>
@@ -1432,7 +1432,7 @@
     <t>Буровий інструмент — це промисловий інструмент, здатний видобувати мінеральні утворення, які інакше непроникні для стандартного спорядження для виживання, без використання костюма Prawn Suit.
 - Посилене промислове алмазне покриття дозволяє руйнувати молекулярні зв'язки великих мінеральних жил.
 - Мікродвигуни, спрямовані назад, запобігають відкиданню оператора назад опором бура.
-- Двигун зі змінним крутним моментом регулює швидкість обертання залежно від щільності матеріалу, щоб запобігти заклинюванню долота та віддачі від перелому зап'ястя.
+- Двигун зі змінним крутним моментом регулює оберти залежно від щільності матеріалу, щоб запобігти заклинюванню долота та віддачі від перелому зап'ястя.
 «Уникаючи необхідності використання важкого транспортного засобу, ви заощадили 4,2 кредити Alterra на амортизації паливних елементів. Будь ласка».</t>
   </si>
   <si>
@@ -1441,6 +1441,257 @@
 - Các động cơ đẩy siêu nhỏ hướng về phía sau ngăn người vận hành bị đẩy lùi do lực cản của mũi khoan
 - Động cơ mô-men xoắn biến đổi điều chỉnh tốc độ quay dựa trên mật độ vật liệu để ngăn ngừa kẹt mũi khoan và hiện tượng giật ngược gây gãy cổ tay
 "Bằng cách bỏ qua nhu cầu sử dụng phương tiện hạng nặng, bạn đã tiết kiệm được cho Alterra 4,2 tín dụng chi phí khấu hao pin nhiên liệu. Không có gì."</t>
+  </si>
+  <si>
+    <t>DrillTool.AutoCollectLabel</t>
+  </si>
+  <si>
+    <t>Auto Collect</t>
+  </si>
+  <si>
+    <t>Outomatiese Versameling</t>
+  </si>
+  <si>
+    <t>Автоматично събиране</t>
+  </si>
+  <si>
+    <t>Recollida automàtica</t>
+  </si>
+  <si>
+    <t>自动收集</t>
+  </si>
+  <si>
+    <t>自動收集</t>
+  </si>
+  <si>
+    <t>Automatsko prikupljanje</t>
+  </si>
+  <si>
+    <t>Automatické vyzvednutí</t>
+  </si>
+  <si>
+    <t>Automatisk afhentning</t>
+  </si>
+  <si>
+    <t>Automaatne kogumine</t>
+  </si>
+  <si>
+    <t>Automaattinen nouto</t>
+  </si>
+  <si>
+    <t>Collecte automatique</t>
+  </si>
+  <si>
+    <t>Automatische Abholung</t>
+  </si>
+  <si>
+    <t>Αυτόματη συλλογή</t>
+  </si>
+  <si>
+    <t>Automatikus átvétel</t>
+  </si>
+  <si>
+    <t>Bailiúchán Uathoibríoch</t>
+  </si>
+  <si>
+    <t>Raccolta automatica</t>
+  </si>
+  <si>
+    <t>自動収集</t>
+  </si>
+  <si>
+    <t>자동 수집</t>
+  </si>
+  <si>
+    <t>Automātiska savākšana</t>
+  </si>
+  <si>
+    <t>Automatinis surinkimas</t>
+  </si>
+  <si>
+    <t>Automatisk henting</t>
+  </si>
+  <si>
+    <t>Automatyczne zbieranie</t>
+  </si>
+  <si>
+    <t>Coleta automática</t>
+  </si>
+  <si>
+    <t>Colectare automată</t>
+  </si>
+  <si>
+    <t>Автоматический сбор</t>
+  </si>
+  <si>
+    <t>Аутоматско прикупљање</t>
+  </si>
+  <si>
+    <t>Automatický zber</t>
+  </si>
+  <si>
+    <t>Samodejno zbiranje</t>
+  </si>
+  <si>
+    <t>Automatisk insamling</t>
+  </si>
+  <si>
+    <t>เก็บเงินอัตโนมัติ</t>
+  </si>
+  <si>
+    <t>Otomatik Toplama</t>
+  </si>
+  <si>
+    <t>Автоматичний збір</t>
+  </si>
+  <si>
+    <t>Thu gom tự động</t>
+  </si>
+  <si>
+    <t>DrillTool.AutoCollectTooltip</t>
+  </si>
+  <si>
+    <t>If enabled, then the mined resources will automatically enter the player's inventory, similar to the behaviour of a Prawn Drill Arm.
+Disabled by default.</t>
+  </si>
+  <si>
+    <t>Indien geaktiveer, sal die ontginde hulpbronne outomaties die speler se inventaris binnegaan, soortgelyk aan die gedrag van 'n Garnaleboorarm.
+Standaard gedeaktiveer.</t>
+  </si>
+  <si>
+    <t>Ако е активирано, добитите ресурси автоматично ще влязат в инвентара на играча, подобно на поведението на ръката за сондажи за скариди.
+Деактивирано по подразбиране.</t>
+  </si>
+  <si>
+    <t>Si està activat, els recursos extrets entraran automàticament a l'inventari del jugador, de manera similar al comportament d'un Prawn Drill Arm.
+Desactivat per defecte.</t>
+  </si>
+  <si>
+    <t>启用后，开采出的资源将自动进入玩家的物品栏，类似于虾式钻臂的操作。
+默认禁用。</t>
+  </si>
+  <si>
+    <t>啟用後，開採的資源將自動進入玩家的物品欄，類似蝦式鑽臂的操作。
+預設禁用。</t>
+  </si>
+  <si>
+    <t>Ako je omogućeno, iskopani resursi će automatski ući u inventar igrača, slično ponašanju ruke za bušenje kozica.
+Onemogućeno prema zadanim postavkama.</t>
+  </si>
+  <si>
+    <t>Pokud je tato možnost povolena, vytěžené zdroje se automaticky dostanou do hráčova inventáře, podobně jako se chová rameno pro vrtání krevet.
+Ve výchozím nastavení je tato možnost zakázána.</t>
+  </si>
+  <si>
+    <t>Hvis aktiveret, vil de udvundne ressourcer automatisk blive tilføjet til spillerens inventar, svarende til en rejeborearms opførsel.
+Deaktiveret som standard.</t>
+  </si>
+  <si>
+    <t>Indien ingeschakeld, komen de gewonnen grondstoffen automatisch in de inventaris van de speler terecht, vergelijkbaar met het gedrag van een Prawn Drill Arm.
+Standaard uitgeschakeld.</t>
+  </si>
+  <si>
+    <t>Kui see on lubatud, siis kaevandatud ressursid lisatakse automaatselt mängija inventari, sarnaselt krevetipuurvarda käitumisele.
+Vaikimisi keelatud.</t>
+  </si>
+  <si>
+    <t>Jos käytössä, louhitut resurssit siirtyvät automaattisesti pelaajan tavaraluetteloon samalla tavalla kuin katkarapuporakone.
+Oletusarvoisesti pois käytöstä.</t>
+  </si>
+  <si>
+    <t>Si cette option est activée, les ressources extraites seront automatiquement ajoutées à l'inventaire du joueur, comme le ferait un bras de forage Prawn.
+Désactivée par défaut.</t>
+  </si>
+  <si>
+    <t>Ist diese Option aktiviert, gelangen die abgebauten Ressourcen automatisch in das Inventar des Spielers, ähnlich wie beim Prawn-Bohrarm. Standardmäßig deaktiviert.</t>
+  </si>
+  <si>
+    <t>Εάν είναι ενεργοποιημένη, τότε οι εξορυγμένοι πόροι θα εισέλθουν αυτόματα στο απόθεμα του παίκτη, παρόμοια με τη συμπεριφορά ενός βραχίονα τρυπανιού γαρίδας.
+Απενεργοποιημένο από προεπιλογή.</t>
+  </si>
+  <si>
+    <t>Ha engedélyezve van, akkor a kibányászott erőforrások automatikusan bekerülnek a játékos felszerelésébe, hasonlóan a garnélarák-fúró kar viselkedéséhez.
+Alapértelmezés szerint letiltva.</t>
+  </si>
+  <si>
+    <t>Má tá sé cumasaithe, cuirfear na hacmhainní mianadóireachta isteach i bhfardal an imreora go huathoibríoch, cosúil le hiompar Lámh Druileála Cloicheán.
+Díchumasaithe de réir réamhshocraithe.</t>
+  </si>
+  <si>
+    <t>Se abilitata, le risorse estratte entreranno automaticamente nell'inventario del giocatore, in modo simile al comportamento di un braccio perforatore Prawn.
+Disabilitata per impostazione predefinita.</t>
+  </si>
+  <si>
+    <t>有効にすると、採掘された資源はプラウンドリルアームと同様に、自動的にプレイヤーのインベントリに格納されます。
+デフォルトでは無効になっています。</t>
+  </si>
+  <si>
+    <t>이 기능을 활성화하면 채굴한 자원이 프론 드릴 암처럼 자동으로 플레이어의 인벤토리에 추가됩니다.
+기본적으로 비활성화되어 있습니다.</t>
+  </si>
+  <si>
+    <t>Ja iespējots, iegūtie resursi automātiski nonāks spēlētāja inventārā, līdzīgi kā garneļu urbšanas roka.
+Pēc noklusējuma atspējots.</t>
+  </si>
+  <si>
+    <t>Jei įjungta, iškasti ištekliai automatiškai pateks į žaidėjo inventorių, panašiai kaip krevečių grąžto rankos veikimas.
+Pagal numatytuosius nustatymus išjungta.</t>
+  </si>
+  <si>
+    <t>Hvis aktivert, vil de utvunnede ressursene automatisk bli lagt inn i spillerens inventar, på samme måte som en rekeborearm oppfører seg.
+Deaktivert som standard.</t>
+  </si>
+  <si>
+    <t>Jeśli ta opcja jest włączona, wydobyte surowce automatycznie trafią do ekwipunku gracza, podobnie jak ramię wiertnicze do krewetek.
+Domyślnie wyłączone.</t>
+  </si>
+  <si>
+    <t>Se ativado, os recursos extraídos entrarão automaticamente no inventário do jogador, de forma semelhante ao comportamento do Braço Perfurador do Prawn.
+Desativado por padrão.</t>
+  </si>
+  <si>
+    <t>Dacă este activată, resursele extrase vor intra automat în inventarul jucătorului, similar comportamentului unui braț de foraj pentru creveți.
+Dezactivată în mod implicit.</t>
+  </si>
+  <si>
+    <t>Если эта функция включена, добытые ресурсы будут автоматически попадать в инвентарь игрока, подобно работе буровой установки Prawn Drill Arm.
+По умолчанию отключено.</t>
+  </si>
+  <si>
+    <t>Ако је омогућено, ископани ресурси ће аутоматски ући у инвентар играча, слично понашању руке за бушење шкампа.
+Подразумевано онемогућено.</t>
+  </si>
+  <si>
+    <t>Ak je povolené, vyťažené zdroje sa automaticky dostanú do hráčovho inventára, podobne ako sa správa rameno na vŕtanie kreviet.
+Predvolene vypnuté.</t>
+  </si>
+  <si>
+    <t>Če je omogočeno, bodo izkopani viri samodejno vstopili v igralčev inventar, podobno kot se obnaša roka za vrtanje kozic.
+Privzeto onemogočeno.</t>
+  </si>
+  <si>
+    <t>Si está activada, los recursos extraídos se añadirán automáticamente al inventario del jugador, de forma similar al comportamiento del Brazo Perforador de Gambas.
+Desactivada por defecto.</t>
+  </si>
+  <si>
+    <t>Om aktiverat kommer de utvunna resurserna automatiskt att läggas in i spelarens inventarieförråd, ungefär som en räkborrarm beter sig.
+Inaktiverad som standard.</t>
+  </si>
+  <si>
+    <t>หากเปิดใช้งาน ทรัพยากรที่ขุดได้จะเข้าสู่คลังของผู้เล่นโดยอัตโนมัติ คล้ายกับพฤติกรรมของแขนเจาะกุ้ง
+ปิดใช้งานโดยค่าเริ่มต้น</t>
+  </si>
+  <si>
+    <t>Etkinleştirilirse, çıkarılan kaynaklar, bir Karides Matkap Kolunun davranışına benzer şekilde, otomatik olarak oyuncunun envanterine girer.
+Varsayılan olarak devre dışıdır.</t>
+  </si>
+  <si>
+    <t>Якщо ввімкнено, то видобуті ресурси автоматично потраплятимуть до інвентарю гравця, подібно до поведінки Креветкової бурильної руки.
+За замовчуванням вимкнено.</t>
+  </si>
+  <si>
+    <t>Nếu được kích hoạt, tài nguyên khai thác được sẽ tự động được chuyển vào kho đồ của người chơi, tương tự như hoạt động của Cánh tay khoan tôm.
+Mặc định là tắt.</t>
   </si>
 </sst>
 </file>
@@ -1722,7 +1973,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1791,6 +2042,12 @@
     </xf>
     <xf borderId="15" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
@@ -2612,587 +2869,587 @@
         <v>164</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P5" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q5" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R5" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S5" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T5" s="14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="U5" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="V5" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W5" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="X5" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="Y5" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Z5" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AA5" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AB5" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AC5" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AD5" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AE5" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AF5" s="14" t="s">
         <v>163</v>
       </c>
       <c r="AG5" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AH5" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AI5" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AJ5" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AK5" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AL5" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AM5" s="14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AN5" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="T6" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="W6" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="X6" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z6" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AC6" s="15" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AD6" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AE6" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AF6" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AG6" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AH6" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AI6" s="15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AJ6" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AK6" s="8" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AL6" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AM6" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AN6" s="17" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K7" s="14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N7" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="R7" s="14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="S7" s="14" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="T7" s="14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U7" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="V7" s="14" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="W7" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="X7" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Y7" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="Z7" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AA7" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AB7" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AC7" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AD7" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AE7" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AF7" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG7" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AH7" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AI7" s="15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AJ7" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AK7" s="14" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AL7" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="AM7" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AN7" s="16" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="N8" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P8" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q8" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="R8" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="T8" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="U8" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="V8" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="W8" s="8" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="X8" s="8" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Y8" s="8" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="Z8" s="8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AA8" s="8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="AC8" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="AD8" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AE8" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AF8" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="AG8" s="8" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="AH8" s="8" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="AI8" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="AJ8" s="8" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AK8" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AL8" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AM8" s="8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="AN8" s="17" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="O9" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="P9" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="Q9" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="R9" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="S9" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="T9" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="U9" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="V9" s="14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="W9" s="14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="X9" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Y9" s="14" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="Z9" s="14" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AA9" s="14" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AB9" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AC9" s="14" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="AD9" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AE9" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AF9" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="AG9" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="AH9" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AI9" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AJ9" s="14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="AK9" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AL9" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AM9" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AN9" s="16" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>40</v>
@@ -3249,7 +3506,7 @@
         <v>40</v>
       </c>
       <c r="T10" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="U10" s="8" t="s">
         <v>40</v>
@@ -3314,124 +3571,124 @@
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N11" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O11" s="14" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="P11" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q11" s="14" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="R11" s="14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="S11" s="14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="T11" s="14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U11" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="V11" s="14" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="W11" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="X11" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Y11" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="Z11" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AA11" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AB11" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AC11" s="14" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AD11" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AE11" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AF11" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG11" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AH11" s="14" t="s">
-        <v>351</v>
+        <v>260</v>
       </c>
       <c r="AI11" s="14" t="s">
-        <v>351</v>
+        <v>260</v>
       </c>
       <c r="AJ11" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AK11" s="14" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AL11" s="14" t="s">
         <v>352</v>
       </c>
       <c r="AM11" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AN11" s="16" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
@@ -3557,349 +3814,547 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="23"/>
-      <c r="Q13" s="23"/>
-      <c r="R13" s="23"/>
-      <c r="S13" s="23"/>
-      <c r="T13" s="23"/>
-      <c r="U13" s="23"/>
+      <c r="A13" s="23" t="s">
+        <v>390</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>391</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>392</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>393</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>394</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>395</v>
+      </c>
+      <c r="G13" s="23" t="s">
+        <v>396</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>397</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>398</v>
+      </c>
+      <c r="J13" s="23" t="s">
+        <v>399</v>
+      </c>
+      <c r="K13" s="23" t="s">
+        <v>391</v>
+      </c>
+      <c r="L13" s="23" t="s">
+        <v>400</v>
+      </c>
+      <c r="M13" s="23" t="s">
+        <v>401</v>
+      </c>
+      <c r="N13" s="23" t="s">
+        <v>402</v>
+      </c>
+      <c r="O13" s="23" t="s">
+        <v>403</v>
+      </c>
+      <c r="P13" s="23" t="s">
+        <v>404</v>
+      </c>
+      <c r="Q13" s="23" t="s">
+        <v>405</v>
+      </c>
+      <c r="R13" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="S13" s="23" t="s">
+        <v>407</v>
+      </c>
+      <c r="T13" s="23" t="s">
+        <v>408</v>
+      </c>
+      <c r="U13" s="23" t="s">
+        <v>409</v>
+      </c>
+      <c r="V13" s="24" t="s">
+        <v>410</v>
+      </c>
+      <c r="W13" s="24" t="s">
+        <v>411</v>
+      </c>
+      <c r="X13" s="24" t="s">
+        <v>412</v>
+      </c>
+      <c r="Y13" s="24" t="s">
+        <v>413</v>
+      </c>
+      <c r="Z13" s="24" t="s">
+        <v>414</v>
+      </c>
+      <c r="AA13" s="24" t="s">
+        <v>414</v>
+      </c>
+      <c r="AB13" s="24" t="s">
+        <v>415</v>
+      </c>
+      <c r="AC13" s="24" t="s">
+        <v>416</v>
+      </c>
+      <c r="AD13" s="24" t="s">
+        <v>417</v>
+      </c>
+      <c r="AE13" s="24" t="s">
+        <v>417</v>
+      </c>
+      <c r="AF13" s="24" t="s">
+        <v>418</v>
+      </c>
+      <c r="AG13" s="24" t="s">
+        <v>419</v>
+      </c>
+      <c r="AH13" s="24" t="s">
+        <v>391</v>
+      </c>
+      <c r="AI13" s="24" t="s">
+        <v>391</v>
+      </c>
+      <c r="AJ13" s="24" t="s">
+        <v>420</v>
+      </c>
+      <c r="AK13" s="24" t="s">
+        <v>421</v>
+      </c>
+      <c r="AL13" s="24" t="s">
+        <v>422</v>
+      </c>
+      <c r="AM13" s="24" t="s">
+        <v>423</v>
+      </c>
+      <c r="AN13" s="24" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="23"/>
-      <c r="P14" s="23"/>
-      <c r="Q14" s="23"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="23"/>
-      <c r="T14" s="23"/>
-      <c r="U14" s="23"/>
+      <c r="A14" s="23" t="s">
+        <v>425</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>426</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>427</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>428</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>429</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>430</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>431</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>432</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>433</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>434</v>
+      </c>
+      <c r="K14" s="23" t="s">
+        <v>435</v>
+      </c>
+      <c r="L14" s="23" t="s">
+        <v>436</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>437</v>
+      </c>
+      <c r="N14" s="23" t="s">
+        <v>438</v>
+      </c>
+      <c r="O14" s="23" t="s">
+        <v>439</v>
+      </c>
+      <c r="P14" s="23" t="s">
+        <v>440</v>
+      </c>
+      <c r="Q14" s="23" t="s">
+        <v>441</v>
+      </c>
+      <c r="R14" s="23" t="s">
+        <v>442</v>
+      </c>
+      <c r="S14" s="23" t="s">
+        <v>443</v>
+      </c>
+      <c r="T14" s="23" t="s">
+        <v>444</v>
+      </c>
+      <c r="U14" s="23" t="s">
+        <v>445</v>
+      </c>
+      <c r="V14" s="24" t="s">
+        <v>446</v>
+      </c>
+      <c r="W14" s="24" t="s">
+        <v>447</v>
+      </c>
+      <c r="X14" s="24" t="s">
+        <v>448</v>
+      </c>
+      <c r="Y14" s="24" t="s">
+        <v>449</v>
+      </c>
+      <c r="Z14" s="24" t="s">
+        <v>450</v>
+      </c>
+      <c r="AA14" s="24" t="s">
+        <v>450</v>
+      </c>
+      <c r="AB14" s="24" t="s">
+        <v>451</v>
+      </c>
+      <c r="AC14" s="24" t="s">
+        <v>452</v>
+      </c>
+      <c r="AD14" s="24" t="s">
+        <v>453</v>
+      </c>
+      <c r="AE14" s="24" t="s">
+        <v>453</v>
+      </c>
+      <c r="AF14" s="24" t="s">
+        <v>454</v>
+      </c>
+      <c r="AG14" s="24" t="s">
+        <v>455</v>
+      </c>
+      <c r="AH14" s="24" t="s">
+        <v>456</v>
+      </c>
+      <c r="AI14" s="24" t="s">
+        <v>456</v>
+      </c>
+      <c r="AJ14" s="24" t="s">
+        <v>457</v>
+      </c>
+      <c r="AK14" s="24" t="s">
+        <v>458</v>
+      </c>
+      <c r="AL14" s="24" t="s">
+        <v>459</v>
+      </c>
+      <c r="AM14" s="24" t="s">
+        <v>460</v>
+      </c>
+      <c r="AN14" s="24" t="s">
+        <v>461</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="23"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="23"/>
-      <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
-      <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
-      <c r="U15" s="23"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="25"/>
+      <c r="M15" s="25"/>
+      <c r="N15" s="25"/>
+      <c r="O15" s="25"/>
+      <c r="P15" s="25"/>
+      <c r="Q15" s="25"/>
+      <c r="R15" s="25"/>
+      <c r="S15" s="25"/>
+      <c r="T15" s="25"/>
+      <c r="U15" s="25"/>
     </row>
     <row r="16">
-      <c r="A16" s="23"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
+      <c r="Q16" s="25"/>
+      <c r="R16" s="25"/>
+      <c r="S16" s="25"/>
+      <c r="T16" s="25"/>
+      <c r="U16" s="25"/>
     </row>
     <row r="17">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
-      <c r="P17" s="23"/>
-      <c r="Q17" s="23"/>
-      <c r="R17" s="23"/>
-      <c r="S17" s="23"/>
-      <c r="T17" s="23"/>
-      <c r="U17" s="23"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
+      <c r="Q17" s="25"/>
+      <c r="R17" s="25"/>
+      <c r="S17" s="25"/>
+      <c r="T17" s="25"/>
+      <c r="U17" s="25"/>
     </row>
     <row r="18">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="23"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
-      <c r="O18" s="23"/>
-      <c r="P18" s="23"/>
-      <c r="Q18" s="23"/>
-      <c r="R18" s="23"/>
-      <c r="S18" s="23"/>
-      <c r="T18" s="23"/>
-      <c r="U18" s="23"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="25"/>
+      <c r="M18" s="25"/>
+      <c r="N18" s="25"/>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
+      <c r="Q18" s="25"/>
+      <c r="R18" s="25"/>
+      <c r="S18" s="25"/>
+      <c r="T18" s="25"/>
+      <c r="U18" s="25"/>
     </row>
     <row r="19">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="23"/>
-      <c r="Q19" s="23"/>
-      <c r="R19" s="23"/>
-      <c r="S19" s="23"/>
-      <c r="T19" s="23"/>
-      <c r="U19" s="23"/>
+      <c r="A19" s="25"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="25"/>
+      <c r="M19" s="25"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
+      <c r="Q19" s="25"/>
+      <c r="R19" s="25"/>
+      <c r="S19" s="25"/>
+      <c r="T19" s="25"/>
+      <c r="U19" s="25"/>
     </row>
     <row r="20">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="23"/>
-      <c r="N20" s="23"/>
-      <c r="O20" s="23"/>
-      <c r="P20" s="23"/>
-      <c r="Q20" s="23"/>
-      <c r="R20" s="23"/>
-      <c r="S20" s="23"/>
-      <c r="T20" s="23"/>
-      <c r="U20" s="23"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="25"/>
+      <c r="M20" s="25"/>
+      <c r="N20" s="25"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
+      <c r="Q20" s="25"/>
+      <c r="R20" s="25"/>
+      <c r="S20" s="25"/>
+      <c r="T20" s="25"/>
+      <c r="U20" s="25"/>
     </row>
     <row r="21">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="23"/>
-      <c r="K21" s="23"/>
-      <c r="L21" s="23"/>
-      <c r="M21" s="23"/>
-      <c r="N21" s="23"/>
-      <c r="O21" s="23"/>
-      <c r="P21" s="23"/>
-      <c r="Q21" s="23"/>
-      <c r="R21" s="23"/>
-      <c r="S21" s="23"/>
-      <c r="T21" s="23"/>
-      <c r="U21" s="23"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="25"/>
+      <c r="L21" s="25"/>
+      <c r="M21" s="25"/>
+      <c r="N21" s="25"/>
+      <c r="O21" s="25"/>
+      <c r="P21" s="25"/>
+      <c r="Q21" s="25"/>
+      <c r="R21" s="25"/>
+      <c r="S21" s="25"/>
+      <c r="T21" s="25"/>
+      <c r="U21" s="25"/>
     </row>
     <row r="22">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="23"/>
-      <c r="K22" s="23"/>
-      <c r="L22" s="23"/>
-      <c r="M22" s="23"/>
-      <c r="N22" s="23"/>
-      <c r="O22" s="23"/>
-      <c r="P22" s="23"/>
-      <c r="Q22" s="23"/>
-      <c r="R22" s="23"/>
-      <c r="S22" s="23"/>
-      <c r="T22" s="23"/>
-      <c r="U22" s="23"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="25"/>
+      <c r="M22" s="25"/>
+      <c r="N22" s="25"/>
+      <c r="O22" s="25"/>
+      <c r="P22" s="25"/>
+      <c r="Q22" s="25"/>
+      <c r="R22" s="25"/>
+      <c r="S22" s="25"/>
+      <c r="T22" s="25"/>
+      <c r="U22" s="25"/>
     </row>
     <row r="23">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-      <c r="N23" s="23"/>
-      <c r="O23" s="23"/>
-      <c r="P23" s="23"/>
-      <c r="Q23" s="23"/>
-      <c r="R23" s="23"/>
-      <c r="S23" s="23"/>
-      <c r="T23" s="23"/>
-      <c r="U23" s="23"/>
+      <c r="A23" s="25"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
+      <c r="M23" s="25"/>
+      <c r="N23" s="25"/>
+      <c r="O23" s="25"/>
+      <c r="P23" s="25"/>
+      <c r="Q23" s="25"/>
+      <c r="R23" s="25"/>
+      <c r="S23" s="25"/>
+      <c r="T23" s="25"/>
+      <c r="U23" s="25"/>
     </row>
     <row r="24">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23"/>
-      <c r="H24" s="23"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="23"/>
-      <c r="K24" s="23"/>
-      <c r="L24" s="23"/>
-      <c r="M24" s="23"/>
-      <c r="N24" s="23"/>
-      <c r="O24" s="23"/>
-      <c r="P24" s="23"/>
-      <c r="Q24" s="23"/>
-      <c r="R24" s="23"/>
-      <c r="S24" s="23"/>
-      <c r="T24" s="23"/>
-      <c r="U24" s="23"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="25"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="25"/>
+      <c r="M24" s="25"/>
+      <c r="N24" s="25"/>
+      <c r="O24" s="25"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="25"/>
+      <c r="R24" s="25"/>
+      <c r="S24" s="25"/>
+      <c r="T24" s="25"/>
+      <c r="U24" s="25"/>
     </row>
     <row r="25">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="23"/>
-      <c r="M25" s="23"/>
-      <c r="N25" s="23"/>
-      <c r="O25" s="23"/>
-      <c r="P25" s="23"/>
-      <c r="Q25" s="23"/>
-      <c r="R25" s="23"/>
-      <c r="S25" s="23"/>
-      <c r="T25" s="23"/>
-      <c r="U25" s="23"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="25"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="25"/>
+      <c r="M25" s="25"/>
+      <c r="N25" s="25"/>
+      <c r="O25" s="25"/>
+      <c r="P25" s="25"/>
+      <c r="Q25" s="25"/>
+      <c r="R25" s="25"/>
+      <c r="S25" s="25"/>
+      <c r="T25" s="25"/>
+      <c r="U25" s="25"/>
     </row>
     <row r="26">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="23"/>
-      <c r="L26" s="23"/>
-      <c r="M26" s="23"/>
-      <c r="N26" s="23"/>
-      <c r="O26" s="23"/>
-      <c r="P26" s="23"/>
-      <c r="Q26" s="23"/>
-      <c r="R26" s="23"/>
-      <c r="S26" s="23"/>
-      <c r="T26" s="23"/>
-      <c r="U26" s="23"/>
+      <c r="A26" s="25"/>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="25"/>
+      <c r="K26" s="25"/>
+      <c r="L26" s="25"/>
+      <c r="M26" s="25"/>
+      <c r="N26" s="25"/>
+      <c r="O26" s="25"/>
+      <c r="P26" s="25"/>
+      <c r="Q26" s="25"/>
+      <c r="R26" s="25"/>
+      <c r="S26" s="25"/>
+      <c r="T26" s="25"/>
+      <c r="U26" s="25"/>
     </row>
     <row r="27">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="23"/>
-      <c r="N27" s="23"/>
-      <c r="O27" s="23"/>
-      <c r="P27" s="23"/>
-      <c r="Q27" s="23"/>
-      <c r="R27" s="23"/>
-      <c r="S27" s="23"/>
-      <c r="T27" s="23"/>
-      <c r="U27" s="23"/>
+      <c r="A27" s="25"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="25"/>
+      <c r="M27" s="25"/>
+      <c r="N27" s="25"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="25"/>
+      <c r="R27" s="25"/>
+      <c r="S27" s="25"/>
+      <c r="T27" s="25"/>
+      <c r="U27" s="25"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>